<commit_message>
Is this is still working?
</commit_message>
<xml_diff>
--- a/documentation/excel/Matriz_Roles_Permisos_Red_House.xlsx
+++ b/documentation/excel/Matriz_Roles_Permisos_Red_House.xlsx
@@ -19774,7 +19774,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/__init__.py:24</t>
+          <t>apps/web/src/__init__.py:24</t>
         </is>
       </c>
     </row>
@@ -19806,7 +19806,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -19838,7 +19838,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/dashboard.py</t>
+          <t>apps/web/src/integration/routes/dashboard.py</t>
         </is>
       </c>
     </row>
@@ -19870,7 +19870,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -19902,7 +19902,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -19934,7 +19934,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -19966,7 +19966,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -19998,7 +19998,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/dashboard.py</t>
+          <t>apps/web/src/integration/routes/dashboard.py</t>
         </is>
       </c>
     </row>
@@ -20030,7 +20030,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/common.py</t>
+          <t>apps/web/src/integration/routes/common.py</t>
         </is>
       </c>
     </row>
@@ -20062,7 +20062,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -20094,7 +20094,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/common.py</t>
+          <t>apps/web/src/integration/routes/common.py</t>
         </is>
       </c>
     </row>
@@ -20126,7 +20126,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/maintenance.py</t>
+          <t>apps/web/src/integration/maintenance.py</t>
         </is>
       </c>
     </row>
@@ -20158,7 +20158,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/maintenance.py</t>
+          <t>apps/web/src/integration/maintenance.py</t>
         </is>
       </c>
     </row>
@@ -20190,7 +20190,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/common.py</t>
+          <t>apps/web/src/integration/routes/common.py</t>
         </is>
       </c>
     </row>
@@ -20254,7 +20254,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/presentation/templates/login.html</t>
+          <t>apps/web/src/presentation/templates/login.html</t>
         </is>
       </c>
     </row>
@@ -20286,7 +20286,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/__init__.py</t>
+          <t>apps/web/src/integration/__init__.py</t>
         </is>
       </c>
     </row>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Nueva DEMO</t>
+          <t>Nueva</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>apps/web-monolito01/src/integration/routes/__init__.py</t>
+          <t>apps/web/src/integration/routes/__init__.py</t>
         </is>
       </c>
     </row>
@@ -20372,7 +20372,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Lanzador integrado, reinicio de un servicio o solo web, datos privados en .local/demo.</t>
+          <t>Lanzador integrado, reinicio de un servicio o solo web, datos privados en .local/runtime.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">

</xml_diff>